<commit_message>
subido EL MIRADOR - PARCIAL
</commit_message>
<xml_diff>
--- a/EL MIRADOR/Agosto/Agosto - EL MIRADOR .xlsx
+++ b/EL MIRADOR/Agosto/Agosto - EL MIRADOR .xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\RC CONSORCIO 2025\EL MIRADOR\Julio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\EL MIRADOR\Agosto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F3FABA-1190-43E9-8AFB-0F7AB8B8D2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5824A098-76BF-42A8-A1BB-17DA230A72A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -858,12 +858,6 @@
 </t>
   </si>
   <si>
-    <t>PERÍODO: JULIO</t>
-  </si>
-  <si>
-    <t>ADS - Abono de mantenimiento ascensores JULIO del 2025</t>
-  </si>
-  <si>
     <t>COCHERA 33</t>
   </si>
   <si>
@@ -921,12 +915,6 @@
     <t>Loschi - Provision bomba electrica para carga de combustible</t>
   </si>
   <si>
-    <t>Articulos de limpieza - Mes de Junio</t>
-  </si>
-  <si>
-    <t>Articulos de limpieza - Mes de Julio</t>
-  </si>
-  <si>
     <t>Metrogas - Cliente nro. 40000496339</t>
   </si>
   <si>
@@ -996,9 +984,6 @@
     <t>Transf 05/07</t>
   </si>
   <si>
-    <t>VTO 14/08</t>
-  </si>
-  <si>
     <t>TOTAL A ABONAR 2DO VTO - DESDE EL</t>
   </si>
   <si>
@@ -1054,6 +1039,21 @@
   </si>
   <si>
     <t xml:space="preserve"> Laura Quintas Perez</t>
+  </si>
+  <si>
+    <t>VTO 15/09</t>
+  </si>
+  <si>
+    <t>PERÍODO: AGOSTO</t>
+  </si>
+  <si>
+    <t>ADS - Abono de mantenimiento ascensores AGOSTO del 2025</t>
+  </si>
+  <si>
+    <t>Articulos de limpieza - Mes de AGOSTO</t>
+  </si>
+  <si>
+    <t>Articulos de limpieza - Mes de JULIO</t>
   </si>
 </sst>
 </file>
@@ -1061,14 +1061,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;\ #,##0;[Red]\-&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;\ #,##0.00;[Red]\-&quot;$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0;[Red]\-&quot;$&quot;\ #,##0"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;\ #,##0.00;[Red]\-&quot;$&quot;\ #,##0.00"/>
-    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_ &quot;$&quot;\ * #,##0.00_ ;_ &quot;$&quot;\ * \-#,##0.00_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
-    <numFmt numFmtId="170" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_ &quot;$&quot;\ * #,##0.00_ ;_ &quot;$&quot;\ * \-#,##0.00_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -1645,8 +1645,8 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="210">
@@ -1658,7 +1658,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1666,95 +1666,95 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="2" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="6" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1763,19 +1763,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="11" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1784,8 +1784,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="10" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="10" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -1799,12 +1799,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="8" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="8" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1815,7 +1815,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1827,13 +1827,13 @@
     <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="8" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="2" fillId="8" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1843,22 +1843,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="11" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="11" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1867,9 +1867,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="16" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1905,14 +1905,26 @@
     <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1920,10 +1932,10 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1946,18 +1958,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2386,23 +2386,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R155"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" customWidth="1"/>
-    <col min="2" max="2" width="36.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="33.44140625" customWidth="1"/>
+    <col min="2" max="2" width="36.88671875" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" customWidth="1"/>
+    <col min="11" max="11" width="15.88671875" customWidth="1"/>
+    <col min="12" max="12" width="16.109375" customWidth="1"/>
     <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="18.28515625" customWidth="1"/>
+    <col min="17" max="17" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="129"/>
       <c r="B1" s="139"/>
       <c r="C1" s="150" t="s">
@@ -2416,7 +2416,7 @@
       <c r="I1" s="127"/>
       <c r="J1" s="128"/>
     </row>
-    <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="130"/>
       <c r="B2" s="140"/>
       <c r="C2" s="140" t="s">
@@ -2430,7 +2430,7 @@
       <c r="I2" s="141"/>
       <c r="J2" s="126"/>
     </row>
-    <row r="3" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="130"/>
       <c r="B3" s="140"/>
       <c r="C3" s="140" t="s">
@@ -2446,7 +2446,7 @@
       <c r="I3" s="141"/>
       <c r="J3" s="126"/>
     </row>
-    <row r="4" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="130"/>
       <c r="B4" s="140"/>
       <c r="C4" s="140" t="s">
@@ -2460,11 +2460,11 @@
       <c r="I4" s="141"/>
       <c r="J4" s="126"/>
     </row>
-    <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="135"/>
       <c r="B5" s="140"/>
       <c r="C5" s="140" t="s">
-        <v>276</v>
+        <v>338</v>
       </c>
       <c r="D5" s="140"/>
       <c r="E5" s="140" t="s">
@@ -2476,7 +2476,7 @@
       <c r="I5" s="140"/>
       <c r="J5" s="136"/>
     </row>
-    <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="135"/>
       <c r="B6" s="140"/>
       <c r="C6" s="140" t="s">
@@ -2490,7 +2490,7 @@
       <c r="I6" s="140"/>
       <c r="J6" s="136"/>
     </row>
-    <row r="7" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="137"/>
       <c r="B7" s="138"/>
       <c r="C7" s="138"/>
@@ -2502,11 +2502,11 @@
       <c r="I7" s="138"/>
       <c r="J7" s="142"/>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="180" t="s">
         <v>269</v>
       </c>
@@ -2520,7 +2520,7 @@
       <c r="I14" s="180"/>
       <c r="J14" s="180"/>
     </row>
-    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="180"/>
       <c r="B15" s="180"/>
       <c r="C15" s="180"/>
@@ -2532,7 +2532,7 @@
       <c r="I15" s="180"/>
       <c r="J15" s="180"/>
     </row>
-    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="180"/>
       <c r="B16" s="180"/>
       <c r="C16" s="180"/>
@@ -2544,7 +2544,7 @@
       <c r="I16" s="180"/>
       <c r="J16" s="180"/>
     </row>
-    <row r="17" spans="1:10" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="180"/>
       <c r="B17" s="180"/>
       <c r="C17" s="180"/>
@@ -2556,7 +2556,7 @@
       <c r="I17" s="180"/>
       <c r="J17" s="180"/>
     </row>
-    <row r="18" spans="1:10" ht="47.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="180"/>
       <c r="B18" s="180"/>
       <c r="C18" s="180"/>
@@ -2568,13 +2568,13 @@
       <c r="I18" s="180"/>
       <c r="J18" s="180"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="H19" s="111"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="190" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B20" s="190"/>
       <c r="C20" s="190"/>
@@ -2586,7 +2586,7 @@
       <c r="I20" s="190"/>
       <c r="J20" s="190"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -2598,7 +2598,7 @@
       <c r="I21" s="190"/>
       <c r="J21" s="190"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="190"/>
       <c r="B22" s="190"/>
       <c r="C22" s="190"/>
@@ -2610,10 +2610,10 @@
       <c r="I22" s="190"/>
       <c r="J22" s="190"/>
     </row>
-    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H23" s="111"/>
     </row>
-    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>20</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="51" t="s">
         <v>241</v>
       </c>
@@ -2653,7 +2653,7 @@
       <c r="I25" s="112"/>
       <c r="J25" s="112"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>46</v>
       </c>
@@ -2669,7 +2669,7 @@
       <c r="I26" s="63"/>
       <c r="J26" s="63"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>244</v>
       </c>
@@ -2685,7 +2685,7 @@
       <c r="I27" s="63"/>
       <c r="J27" s="63"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>242</v>
       </c>
@@ -2701,7 +2701,7 @@
       <c r="I28" s="63"/>
       <c r="J28" s="63"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>243</v>
       </c>
@@ -2717,7 +2717,7 @@
       <c r="I29" s="63"/>
       <c r="J29" s="63"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>245</v>
       </c>
@@ -2733,7 +2733,7 @@
       <c r="I30" s="63"/>
       <c r="J30" s="63"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="110" t="s">
         <v>172</v>
       </c>
@@ -2750,7 +2750,7 @@
       <c r="I31" s="109"/>
       <c r="J31" s="109"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="51" t="s">
         <v>240</v>
       </c>
@@ -2764,7 +2764,7 @@
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>46</v>
       </c>
@@ -2780,7 +2780,7 @@
       <c r="I33" s="63"/>
       <c r="J33" s="63"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>244</v>
       </c>
@@ -2796,7 +2796,7 @@
       <c r="I34" s="63"/>
       <c r="J34" s="63"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>242</v>
       </c>
@@ -2812,7 +2812,7 @@
       <c r="I35" s="63"/>
       <c r="J35" s="63"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>243</v>
       </c>
@@ -2828,7 +2828,7 @@
       <c r="I36" s="63"/>
       <c r="J36" s="63"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>245</v>
       </c>
@@ -2844,7 +2844,7 @@
       <c r="I37" s="63"/>
       <c r="J37" s="63"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="110" t="s">
         <v>172</v>
       </c>
@@ -2861,7 +2861,7 @@
       <c r="I38" s="109"/>
       <c r="J38" s="109"/>
     </row>
-    <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="34" t="s">
         <v>1</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33" t="s">
         <v>35</v>
       </c>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="L40" s="74"/>
     </row>
-    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="33"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="L41" s="74"/>
     </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="33"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -2961,7 +2961,7 @@
       <c r="J42" s="6"/>
       <c r="L42" s="74"/>
     </row>
-    <row r="43" spans="1:12" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" ht="0.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="33"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -2974,7 +2974,7 @@
       <c r="J43" s="6"/>
       <c r="L43" s="74"/>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="34" t="s">
         <v>41</v>
       </c>
@@ -3005,7 +3005,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="33" t="s">
         <v>256</v>
       </c>
@@ -3026,13 +3026,13 @@
       </c>
       <c r="L45" s="74"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>257</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D46" s="96">
         <v>37011.99</v>
@@ -3048,13 +3048,13 @@
       <c r="J46" s="63"/>
       <c r="L46" s="74"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>257</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="6" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D47" s="96">
         <v>65006.06</v>
@@ -3070,13 +3070,13 @@
       <c r="J47" s="63"/>
       <c r="L47" s="74"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>257</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D48" s="96">
         <v>26019.040000000001</v>
@@ -3092,13 +3092,13 @@
       <c r="J48" s="63"/>
       <c r="L48" s="74"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>257</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D49" s="96">
         <v>23000</v>
@@ -3114,13 +3114,13 @@
       <c r="J49" s="63"/>
       <c r="L49" s="74"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>257</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D50" s="96">
         <v>27002.95</v>
@@ -3136,7 +3136,7 @@
       <c r="J50" s="63"/>
       <c r="L50" s="74"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="33"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="L51" s="74"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="34" t="s">
         <v>36</v>
       </c>
@@ -3183,7 +3183,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="33" t="s">
         <v>250</v>
       </c>
@@ -3198,7 +3198,7 @@
       <c r="J53" s="50"/>
       <c r="L53" s="74"/>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="36" t="s">
         <v>253</v>
       </c>
@@ -3213,13 +3213,13 @@
       <c r="J54" s="50"/>
       <c r="L54" s="74"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="36" t="s">
         <v>255</v>
       </c>
       <c r="B55" s="36"/>
       <c r="C55" s="36" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D55" s="96">
         <v>643422</v>
@@ -3232,13 +3232,13 @@
       <c r="J55" s="50"/>
       <c r="L55" s="74"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56" s="36" t="s">
         <v>254</v>
       </c>
       <c r="B56" s="36"/>
       <c r="C56" s="36" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D56" s="96">
         <v>643422</v>
@@ -3251,7 +3251,7 @@
       <c r="J56" s="50"/>
       <c r="L56" s="74"/>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" s="34" t="s">
         <v>252</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="33" t="s">
         <v>2</v>
       </c>
@@ -3309,13 +3309,13 @@
       <c r="J58" s="6"/>
       <c r="L58" s="74"/>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
         <v>246</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="6" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D59" s="45">
         <v>49257.04</v>
@@ -3328,13 +3328,13 @@
       <c r="J59" s="6"/>
       <c r="L59" s="74"/>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="6" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D60" s="45">
         <v>56422.63</v>
@@ -3347,7 +3347,7 @@
       <c r="J60" s="6"/>
       <c r="L60" s="74"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="34" t="s">
         <v>251</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="33" t="s">
         <v>233</v>
       </c>
@@ -3405,13 +3405,13 @@
       <c r="J62" s="37"/>
       <c r="L62" s="74"/>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
         <v>237</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D63" s="45">
         <v>160913</v>
@@ -3446,13 +3446,13 @@
       </c>
       <c r="L63" s="74"/>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>238</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D64" s="45">
         <v>7907</v>
@@ -3487,13 +3487,13 @@
       </c>
       <c r="L64" s="74"/>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>239</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D65" s="45">
         <v>7907</v>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="L65" s="74"/>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="34" t="s">
         <v>3</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="33" t="s">
         <v>4</v>
       </c>
@@ -3586,13 +3586,13 @@
       <c r="J67" s="6"/>
       <c r="L67" s="74"/>
     </row>
-    <row r="68" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="79" t="s">
         <v>247</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D68" s="147">
         <v>161756.56</v>
@@ -3638,13 +3638,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>248</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D69" s="147">
         <v>1233986.03</v>
@@ -3690,13 +3690,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>249</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="6" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D70" s="45">
         <v>100525.5</v>
@@ -3727,13 +3727,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
-        <v>277</v>
+        <v>339</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="6" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D71" s="45">
         <v>263223.14</v>
@@ -3758,9 +3758,9 @@
       <c r="M71" s="95"/>
       <c r="N71" s="95"/>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="36" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B72" s="36"/>
       <c r="C72" s="36"/>
@@ -3793,13 +3793,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" s="36" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B73" s="36"/>
       <c r="C73" s="36" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D73" s="45">
         <v>25666.87</v>
@@ -3845,13 +3845,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="36" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B74" s="36"/>
       <c r="C74" s="36" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D74" s="45">
         <v>32660.43</v>
@@ -3897,9 +3897,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="79" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B75" s="132"/>
       <c r="C75" s="132"/>
@@ -3932,9 +3932,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="173" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B76" s="173"/>
       <c r="C76" s="174"/>
@@ -3967,7 +3967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="79"/>
       <c r="B77" s="80"/>
       <c r="C77" s="80"/>
@@ -3985,7 +3985,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="34" t="s">
         <v>5</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="6"/>
@@ -4045,7 +4045,7 @@
       <c r="J79" s="6"/>
       <c r="L79" s="74"/>
     </row>
-    <row r="80" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="6"/>
@@ -4058,7 +4058,7 @@
       <c r="J80" s="6"/>
       <c r="L80" s="74"/>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="33" t="s">
         <v>234</v>
       </c>
@@ -4073,9 +4073,9 @@
       <c r="J81" s="6"/>
       <c r="L81" s="74"/>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
-        <v>297</v>
+        <v>341</v>
       </c>
       <c r="B82" s="36"/>
       <c r="C82" s="6"/>
@@ -4110,9 +4110,9 @@
       <c r="K82" s="82"/>
       <c r="L82" s="74"/>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
-        <v>298</v>
+        <v>340</v>
       </c>
       <c r="B83" s="36"/>
       <c r="C83" s="6"/>
@@ -4146,9 +4146,9 @@
       <c r="K83" s="82"/>
       <c r="L83" s="74"/>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="B84" s="36"/>
       <c r="C84" s="6"/>
@@ -4182,9 +4182,9 @@
       <c r="K84" s="82"/>
       <c r="L84" s="74"/>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B85" s="36"/>
       <c r="C85" s="6"/>
@@ -4218,9 +4218,9 @@
       <c r="K85" s="82"/>
       <c r="L85" s="74"/>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B86" s="36"/>
       <c r="C86" s="6"/>
@@ -4254,9 +4254,9 @@
       <c r="K86" s="82"/>
       <c r="L86" s="74"/>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B87" s="36"/>
       <c r="C87" s="6"/>
@@ -4275,7 +4275,7 @@
       <c r="K87" s="82"/>
       <c r="L87" s="74"/>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6"/>
@@ -4289,7 +4289,7 @@
       <c r="L88" s="74"/>
       <c r="M88" s="44"/>
     </row>
-    <row r="89" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="34" t="s">
         <v>235</v>
       </c>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="N89" s="44"/>
     </row>
-    <row r="90" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="6"/>
@@ -4346,7 +4346,7 @@
       <c r="J90" s="6"/>
       <c r="L90" s="74"/>
     </row>
-    <row r="91" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="6"/>
       <c r="B91" s="6"/>
       <c r="C91" s="6"/>
@@ -4359,7 +4359,7 @@
       <c r="J91" s="6"/>
       <c r="L91" s="74"/>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" s="33" t="s">
         <v>6</v>
       </c>
@@ -4374,7 +4374,7 @@
       <c r="J92" s="6"/>
       <c r="L92" s="74"/>
     </row>
-    <row r="93" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>7</v>
       </c>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="L93" s="74"/>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" s="33"/>
       <c r="B94" s="6"/>
       <c r="C94" s="6"/>
@@ -4425,7 +4425,7 @@
       <c r="L94" s="74"/>
       <c r="N94" s="45"/>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="6"/>
@@ -4439,7 +4439,7 @@
       <c r="L95" s="74"/>
       <c r="N95" s="44"/>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" s="34" t="s">
         <v>8</v>
       </c>
@@ -4483,12 +4483,12 @@
       </c>
       <c r="N96" s="44"/>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C97" s="6"/>
       <c r="D97" s="45"/>
@@ -4518,12 +4518,12 @@
       </c>
       <c r="L97" s="74"/>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C98" s="52"/>
       <c r="D98" s="45"/>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="L98" s="74"/>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" s="34" t="s">
         <v>236</v>
       </c>
@@ -4596,7 +4596,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="115"/>
       <c r="B100" s="115"/>
       <c r="C100" s="115"/>
@@ -4609,7 +4609,7 @@
       <c r="J100" s="115"/>
       <c r="L100" s="74"/>
     </row>
-    <row r="101" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A101" s="117" t="s">
         <v>47</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A102" s="120"/>
       <c r="B102" s="121"/>
       <c r="C102" s="121"/>
@@ -4665,7 +4665,7 @@
       <c r="K102" s="44"/>
       <c r="L102" s="74"/>
     </row>
-    <row r="103" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
         <v>31</v>
       </c>
@@ -4712,7 +4712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D104" s="98"/>
       <c r="E104" s="44"/>
       <c r="F104" s="44"/>
@@ -4720,7 +4720,7 @@
       <c r="H104" s="44"/>
       <c r="I104" s="44"/>
     </row>
-    <row r="105" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A105" s="69" t="s">
         <v>42</v>
       </c>
@@ -4732,9 +4732,9 @@
       <c r="H105" s="44"/>
       <c r="I105" s="44"/>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="C106" s="149">
         <f>21780*2</f>
@@ -4746,9 +4746,9 @@
       <c r="H106" s="44"/>
       <c r="I106" s="44"/>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="C107" s="149">
         <v>21780</v>
@@ -4759,9 +4759,9 @@
       <c r="H107" s="44"/>
       <c r="I107" s="44"/>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C108" s="149">
         <v>18000</v>
@@ -4772,9 +4772,9 @@
       <c r="H108" s="44"/>
       <c r="I108" s="44"/>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C109" s="149">
         <v>9000</v>
@@ -4785,9 +4785,9 @@
       <c r="H109" s="44"/>
       <c r="I109" s="44"/>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C110" s="149">
         <v>18000</v>
@@ -4798,9 +4798,9 @@
       <c r="H110" s="44"/>
       <c r="I110" s="44"/>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C111" s="149">
         <v>18000</v>
@@ -4811,9 +4811,9 @@
       <c r="H111" s="44"/>
       <c r="I111" s="44"/>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C112" s="149">
         <v>9000</v>
@@ -4824,9 +4824,9 @@
       <c r="H112" s="44"/>
       <c r="I112" s="44"/>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C113" s="149">
         <v>9000</v>
@@ -4837,9 +4837,9 @@
       <c r="H113" s="44"/>
       <c r="I113" s="44"/>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C114" s="149">
         <v>9000</v>
@@ -4850,9 +4850,9 @@
       <c r="H114" s="44"/>
       <c r="I114" s="44"/>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C115" s="149">
         <v>9000</v>
@@ -4863,7 +4863,7 @@
       <c r="H115" s="44"/>
       <c r="I115" s="44"/>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A116" s="1"/>
       <c r="C116" s="175"/>
       <c r="E116" s="44"/>
@@ -4872,7 +4872,7 @@
       <c r="H116" s="44"/>
       <c r="I116" s="44"/>
     </row>
-    <row r="117" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1"/>
       <c r="C117" s="175"/>
       <c r="E117" s="44"/>
@@ -4881,7 +4881,7 @@
       <c r="H117" s="44"/>
       <c r="I117" s="44"/>
     </row>
-    <row r="118" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="70" t="s">
         <v>18</v>
       </c>
@@ -4896,21 +4896,21 @@
       <c r="H118" s="44"/>
       <c r="I118" s="44"/>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E119" s="44"/>
       <c r="F119" s="44"/>
       <c r="G119" s="44"/>
       <c r="H119" s="44"/>
       <c r="I119" s="44"/>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E120" s="65"/>
       <c r="F120" s="65"/>
       <c r="G120" s="65"/>
       <c r="H120" s="65"/>
       <c r="I120" s="65"/>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A121" s="186" t="s">
         <v>37</v>
       </c>
@@ -4936,7 +4936,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="122" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="188"/>
       <c r="B122" s="189"/>
       <c r="C122" s="92"/>
@@ -4951,7 +4951,7 @@
       <c r="I122" s="73"/>
       <c r="J122" s="63"/>
     </row>
-    <row r="123" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="188"/>
       <c r="B123" s="189"/>
       <c r="C123" s="92"/>
@@ -4963,7 +4963,7 @@
       <c r="I123" s="73"/>
       <c r="J123" s="63"/>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A124" s="183" t="s">
         <v>18</v>
       </c>
@@ -4994,14 +4994,14 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E126" s="44"/>
       <c r="F126" s="44"/>
       <c r="G126" s="44"/>
       <c r="H126" s="44"/>
       <c r="I126" s="44"/>
     </row>
-    <row r="127" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A127" s="39" t="s">
         <v>32</v>
       </c>
@@ -5010,7 +5010,7 @@
         <v>9142586.040000001</v>
       </c>
     </row>
-    <row r="128" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A128" s="41" t="s">
         <v>34</v>
       </c>
@@ -5019,7 +5019,7 @@
         <v>7642586.040000001</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D129" s="182"/>
       <c r="E129" s="182"/>
       <c r="F129" s="102"/>
@@ -5027,7 +5027,7 @@
       <c r="H129" s="102"/>
       <c r="I129" s="102"/>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130" s="17" t="s">
         <v>21</v>
       </c>
@@ -5040,7 +5040,7 @@
       <c r="H130" s="102"/>
       <c r="I130" s="102"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" s="20" t="s">
         <v>22</v>
       </c>
@@ -5055,7 +5055,7 @@
       <c r="H131" s="102"/>
       <c r="I131" s="102"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="22" t="s">
         <v>23</v>
       </c>
@@ -5073,7 +5073,7 @@
       <c r="H132" s="102"/>
       <c r="I132" s="102"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133" s="22" t="s">
         <v>39</v>
       </c>
@@ -5090,7 +5090,7 @@
       <c r="I133" s="102"/>
       <c r="K133" s="45"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134" s="22" t="s">
         <v>38</v>
       </c>
@@ -5107,7 +5107,7 @@
       <c r="I134" s="102"/>
       <c r="K134" s="55"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135" s="22" t="s">
         <v>33</v>
       </c>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="C135" s="23"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136" s="22" t="s">
         <v>42</v>
       </c>
@@ -5127,12 +5127,12 @@
       </c>
       <c r="C136" s="23"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137" s="22"/>
       <c r="B137" s="18"/>
       <c r="C137" s="23"/>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138" s="20" t="s">
         <v>25</v>
       </c>
@@ -5142,12 +5142,12 @@
       </c>
       <c r="C138" s="78"/>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A139" s="23"/>
       <c r="C139" s="19"/>
       <c r="D139" s="26"/>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C140" s="19"/>
       <c r="D140" s="44"/>
       <c r="E140" s="95"/>
@@ -5156,7 +5156,7 @@
       <c r="H140" s="95"/>
       <c r="I140" s="95"/>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141" s="17" t="s">
         <v>26</v>
       </c>
@@ -5172,7 +5172,7 @@
       <c r="I141" s="95"/>
       <c r="J141" s="95"/>
     </row>
-    <row r="142" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="20" t="s">
         <v>264</v>
       </c>
@@ -5185,7 +5185,7 @@
       <c r="H142" s="103"/>
       <c r="I142" s="103"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" s="20"/>
       <c r="B143" s="94"/>
       <c r="C143" s="25"/>
@@ -5195,7 +5195,7 @@
       <c r="H143" s="44"/>
       <c r="I143" s="44"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="37" t="s">
         <v>18</v>
       </c>
@@ -5205,18 +5205,18 @@
       </c>
       <c r="C144" s="25"/>
     </row>
-    <row r="145" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:18" x14ac:dyDescent="0.3">
       <c r="C145" s="26"/>
       <c r="D145" s="95"/>
     </row>
-    <row r="146" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B146" s="23"/>
       <c r="C146" s="19"/>
     </row>
-    <row r="148" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:18" x14ac:dyDescent="0.3">
       <c r="R148" s="10"/>
     </row>
-    <row r="151" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B151" s="181"/>
       <c r="C151" s="181"/>
       <c r="D151" s="181"/>
@@ -5226,7 +5226,7 @@
       <c r="H151" s="106"/>
       <c r="I151" s="106"/>
     </row>
-    <row r="152" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B152" s="181"/>
       <c r="C152" s="181"/>
       <c r="D152" s="181"/>
@@ -5236,7 +5236,7 @@
       <c r="H152" s="106"/>
       <c r="I152" s="106"/>
     </row>
-    <row r="153" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B153" s="181"/>
       <c r="C153" s="181"/>
       <c r="D153" s="181"/>
@@ -5246,7 +5246,7 @@
       <c r="H153" s="106"/>
       <c r="I153" s="106"/>
     </row>
-    <row r="154" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B154" s="181"/>
       <c r="C154" s="181"/>
       <c r="D154" s="181"/>
@@ -5256,7 +5256,7 @@
       <c r="H154" s="106"/>
       <c r="I154" s="106"/>
     </row>
-    <row r="155" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B155" s="181"/>
       <c r="C155" s="181"/>
       <c r="D155" s="181"/>
@@ -5286,27 +5286,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R148"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="5.85546875" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="8.140625" customWidth="1"/>
-    <col min="4" max="4" width="43.5703125" customWidth="1"/>
-    <col min="5" max="5" width="39.7109375" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" customWidth="1"/>
+    <col min="4" max="4" width="43.5546875" customWidth="1"/>
+    <col min="5" max="5" width="39.6640625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
     <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.28515625" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" customWidth="1"/>
-    <col min="14" max="14" width="13.7109375" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" customWidth="1"/>
-    <col min="16" max="16" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.33203125" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" customWidth="1"/>
+    <col min="14" max="14" width="13.6640625" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" customWidth="1"/>
+    <col min="16" max="16" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -5322,15 +5322,15 @@
       <c r="K1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="L1" s="196">
+      <c r="L1" s="200">
         <f>RESUMEN!D103-RESUMEN!D101</f>
         <v>7642586.040000001</v>
       </c>
-      <c r="M1" s="197"/>
+      <c r="M1" s="201"/>
       <c r="N1" s="76"/>
       <c r="O1" s="64"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -5351,10 +5351,10 @@
       <c r="N2" s="77"/>
       <c r="O2" s="64"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="str">
         <f>RESUMEN!C5</f>
-        <v>PERÍODO: JULIO</v>
+        <v>PERÍODO: AGOSTO</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -5371,7 +5371,7 @@
       <c r="N3" s="75"/>
       <c r="O3" s="16"/>
     </row>
-    <row r="4" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -5394,89 +5394,89 @@
         <v>-1240893.8416399993</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="192" t="s">
+    <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="191" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="205" t="s">
+      <c r="B5" s="193" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="192" t="s">
+      <c r="C5" s="191" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="207" t="s">
+      <c r="D5" s="195" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="207" t="s">
-        <v>281</v>
-      </c>
-      <c r="F5" s="192" t="s">
+      <c r="E5" s="195" t="s">
+        <v>279</v>
+      </c>
+      <c r="F5" s="191" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="192" t="s">
+      <c r="G5" s="191" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="192" t="s">
+      <c r="H5" s="191" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="198" t="s">
+      <c r="I5" s="202" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="200" t="s">
+      <c r="J5" s="204" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="200" t="s">
+      <c r="K5" s="204" t="s">
         <v>19</v>
       </c>
-      <c r="L5" s="203" t="s">
+      <c r="L5" s="207" t="s">
         <v>43</v>
       </c>
-      <c r="M5" s="200" t="s">
-        <v>324</v>
-      </c>
-      <c r="N5" s="200" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="193"/>
-      <c r="B6" s="206"/>
-      <c r="C6" s="193"/>
-      <c r="D6" s="208"/>
-      <c r="E6" s="208"/>
-      <c r="F6" s="193"/>
-      <c r="G6" s="193"/>
-      <c r="H6" s="193"/>
-      <c r="I6" s="199"/>
-      <c r="J6" s="201"/>
-      <c r="K6" s="201"/>
-      <c r="L6" s="204"/>
-      <c r="M6" s="201"/>
-      <c r="N6" s="201"/>
-    </row>
-    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="193"/>
-      <c r="B7" s="206"/>
-      <c r="C7" s="193"/>
-      <c r="D7" s="208"/>
-      <c r="E7" s="208"/>
-      <c r="F7" s="193"/>
-      <c r="G7" s="193"/>
-      <c r="H7" s="193"/>
-      <c r="I7" s="199"/>
-      <c r="J7" s="201"/>
-      <c r="K7" s="202"/>
-      <c r="L7" s="204"/>
+      <c r="M5" s="204" t="s">
+        <v>319</v>
+      </c>
+      <c r="N5" s="204" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="192"/>
+      <c r="B6" s="194"/>
+      <c r="C6" s="192"/>
+      <c r="D6" s="196"/>
+      <c r="E6" s="196"/>
+      <c r="F6" s="192"/>
+      <c r="G6" s="192"/>
+      <c r="H6" s="192"/>
+      <c r="I6" s="203"/>
+      <c r="J6" s="205"/>
+      <c r="K6" s="205"/>
+      <c r="L6" s="208"/>
+      <c r="M6" s="205"/>
+      <c r="N6" s="205"/>
+    </row>
+    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="192"/>
+      <c r="B7" s="194"/>
+      <c r="C7" s="192"/>
+      <c r="D7" s="196"/>
+      <c r="E7" s="196"/>
+      <c r="F7" s="192"/>
+      <c r="G7" s="192"/>
+      <c r="H7" s="192"/>
+      <c r="I7" s="203"/>
+      <c r="J7" s="205"/>
+      <c r="K7" s="206"/>
+      <c r="L7" s="208"/>
       <c r="M7" s="153" t="str">
         <f>RESUMEN!A20</f>
-        <v>VTO 14/08</v>
+        <v>VTO 15/09</v>
       </c>
       <c r="N7" s="152" t="str">
         <f>RESUMEN!A20</f>
-        <v>VTO 14/08</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+        <v>VTO 15/09</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>122</v>
       </c>
@@ -5521,12 +5521,12 @@
         <v>86445.848309040011</v>
       </c>
       <c r="O8" s="133"/>
-      <c r="Q8" s="191" t="s">
+      <c r="Q8" s="197" t="s">
         <v>263</v>
       </c>
-      <c r="R8" s="191"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R8" s="197"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6" t="s">
@@ -5569,10 +5569,10 @@
         <v>102454.33873664</v>
       </c>
       <c r="O9" s="133"/>
-      <c r="Q9" s="191"/>
-      <c r="R9" s="191"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q9" s="197"/>
+      <c r="R9" s="197"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>122</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>118</v>
       </c>
       <c r="D10" s="62" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E10" s="62"/>
       <c r="F10" s="105">
@@ -5625,7 +5625,7 @@
         <v>82162.051487999997</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>122</v>
       </c>
@@ -5678,7 +5678,7 @@
         <v>97377.246207999997</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>122</v>
       </c>
@@ -5687,7 +5687,7 @@
         <v>120</v>
       </c>
       <c r="D12" s="169" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E12" s="169"/>
       <c r="F12" s="163">
@@ -5731,7 +5731,7 @@
         <v>92051.928055999975</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="62" t="s">
         <v>124</v>
       </c>
@@ -5788,7 +5788,7 @@
         <v>113353.200664</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="62" t="s">
         <v>125</v>
       </c>
@@ -5845,7 +5845,7 @@
         <v>132372.19406399998</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="62" t="s">
         <v>124</v>
       </c>
@@ -5896,7 +5896,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="62" t="s">
         <v>126</v>
       </c>
@@ -5944,7 +5944,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="62" t="s">
         <v>126</v>
       </c>
@@ -5994,7 +5994,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="62" t="s">
         <v>126</v>
       </c>
@@ -6006,7 +6006,7 @@
         <v>186</v>
       </c>
       <c r="E18" s="172" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F18" s="104">
         <v>9.4999999999999998E-3</v>
@@ -6043,7 +6043,7 @@
         <v>6.0000000000000005E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="62" t="s">
         <v>124</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="62" t="s">
         <v>125</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>55</v>
       </c>
       <c r="D20" s="62" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E20" s="172"/>
       <c r="F20" s="104">
@@ -6142,7 +6142,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="62" t="s">
         <v>124</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="62" t="s">
         <v>126</v>
       </c>
@@ -6241,7 +6241,7 @@
         <v>9.9999999999999992E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="62" t="s">
         <v>126</v>
       </c>
@@ -6292,7 +6292,7 @@
         <v>0.10999999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="62" t="s">
         <v>126</v>
       </c>
@@ -6343,7 +6343,7 @@
         <v>0.11999999999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="62" t="s">
         <v>124</v>
       </c>
@@ -6394,7 +6394,7 @@
         <v>0.12999999999999998</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="62" t="s">
         <v>125</v>
       </c>
@@ -6406,7 +6406,7 @@
         <v>265</v>
       </c>
       <c r="E26" s="172" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F26" s="104">
         <v>7.1999999999999998E-3</v>
@@ -6444,7 +6444,7 @@
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="62" t="s">
         <v>124</v>
       </c>
@@ -6495,7 +6495,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="62" t="s">
         <v>126</v>
       </c>
@@ -6546,7 +6546,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="62" t="s">
         <v>126</v>
       </c>
@@ -6597,7 +6597,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="62" t="s">
         <v>126</v>
       </c>
@@ -6648,7 +6648,7 @@
         <v>0.18000000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="62" t="s">
         <v>124</v>
       </c>
@@ -6699,7 +6699,7 @@
         <v>0.19000000000000003</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="62" t="s">
         <v>125</v>
       </c>
@@ -6750,7 +6750,7 @@
         <v>0.20000000000000004</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" s="62" t="s">
         <v>124</v>
       </c>
@@ -6798,7 +6798,7 @@
         <v>0.21000000000000005</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" s="62" t="s">
         <v>126</v>
       </c>
@@ -6807,7 +6807,7 @@
         <v>69</v>
       </c>
       <c r="D34" s="62" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E34" s="172"/>
       <c r="F34" s="104">
@@ -6849,7 +6849,7 @@
         <v>0.22000000000000006</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="62" t="s">
         <v>126</v>
       </c>
@@ -6900,7 +6900,7 @@
         <v>0.23000000000000007</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" s="62" t="s">
         <v>126</v>
       </c>
@@ -6909,7 +6909,7 @@
         <v>71</v>
       </c>
       <c r="D36" s="62" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E36" s="172"/>
       <c r="F36" s="104">
@@ -6951,7 +6951,7 @@
         <v>0.24000000000000007</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" s="62" t="s">
         <v>124</v>
       </c>
@@ -7002,7 +7002,7 @@
         <v>0.25000000000000006</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" s="62" t="s">
         <v>125</v>
       </c>
@@ -7014,7 +7014,7 @@
         <v>193</v>
       </c>
       <c r="E38" s="172" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F38" s="104">
         <v>7.1999999999999998E-3</v>
@@ -7054,7 +7054,7 @@
         <v>0.26000000000000006</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" s="62" t="s">
         <v>124</v>
       </c>
@@ -7104,13 +7104,13 @@
         <v>0.27000000000000007</v>
       </c>
       <c r="P39" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="Q39" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40" s="62" t="s">
         <v>126</v>
       </c>
@@ -7164,7 +7164,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" s="62" t="s">
         <v>126</v>
       </c>
@@ -7215,7 +7215,7 @@
         <v>0.29000000000000009</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" s="62" t="s">
         <v>126</v>
       </c>
@@ -7266,7 +7266,7 @@
         <v>0.3000000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43" s="62" t="s">
         <v>124</v>
       </c>
@@ -7316,7 +7316,7 @@
         <v>0.31000000000000011</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44" s="62" t="s">
         <v>125</v>
       </c>
@@ -7368,7 +7368,7 @@
       </c>
       <c r="P44" s="44"/>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45" s="62" t="s">
         <v>124</v>
       </c>
@@ -7419,7 +7419,7 @@
       </c>
       <c r="P45" s="44"/>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46" s="62" t="s">
         <v>126</v>
       </c>
@@ -7470,7 +7470,7 @@
         <v>0.34000000000000014</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47" s="62" t="s">
         <v>126</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>0.35000000000000014</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48" s="62" t="s">
         <v>126</v>
       </c>
@@ -7569,7 +7569,7 @@
         <v>0.36000000000000015</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" s="62" t="s">
         <v>124</v>
       </c>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="Q49" s="64"/>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50" s="62" t="s">
         <v>125</v>
       </c>
@@ -7633,7 +7633,7 @@
         <v>201</v>
       </c>
       <c r="E50" s="172" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F50" s="104">
         <v>7.1999999999999998E-3</v>
@@ -7673,7 +7673,7 @@
         <v>0.38000000000000017</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A51" s="62" t="s">
         <v>124</v>
       </c>
@@ -7724,7 +7724,7 @@
         <v>0.39000000000000018</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52" s="62" t="s">
         <v>126</v>
       </c>
@@ -7772,7 +7772,7 @@
         <v>0.40000000000000019</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" s="62" t="s">
         <v>126</v>
       </c>
@@ -7826,7 +7826,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54" s="62" t="s">
         <v>126</v>
       </c>
@@ -7874,10 +7874,10 @@
         <v>0.42000000000000021</v>
       </c>
       <c r="P54" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55" s="62" t="s">
         <v>124</v>
       </c>
@@ -7927,7 +7927,7 @@
         <v>0.43000000000000022</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56" s="62" t="s">
         <v>125</v>
       </c>
@@ -7978,7 +7978,7 @@
         <v>0.44000000000000022</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57" s="62" t="s">
         <v>124</v>
       </c>
@@ -8029,7 +8029,7 @@
         <v>0.45000000000000023</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58" s="62" t="s">
         <v>126</v>
       </c>
@@ -8041,7 +8041,7 @@
         <v>207</v>
       </c>
       <c r="E58" s="172" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="F58" s="104">
         <v>9.4000000000000004E-3</v>
@@ -8079,7 +8079,7 @@
         <v>0.46000000000000024</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59" s="62" t="s">
         <v>126</v>
       </c>
@@ -8129,7 +8129,7 @@
         <v>0.47000000000000025</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A60" s="62" t="s">
         <v>126</v>
       </c>
@@ -8179,7 +8179,7 @@
         <v>0.48000000000000026</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61" s="62" t="s">
         <v>124</v>
       </c>
@@ -8230,7 +8230,7 @@
         <v>0.49000000000000027</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62" s="62" t="s">
         <v>125</v>
       </c>
@@ -8278,7 +8278,7 @@
         <v>0.50000000000000022</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63" s="62" t="s">
         <v>124</v>
       </c>
@@ -8329,7 +8329,7 @@
         <v>0.51000000000000023</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64" s="62" t="s">
         <v>126</v>
       </c>
@@ -8377,7 +8377,7 @@
         <v>0.52000000000000024</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A65" s="62" t="s">
         <v>126</v>
       </c>
@@ -8431,7 +8431,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A66" s="62" t="s">
         <v>126</v>
       </c>
@@ -8482,7 +8482,7 @@
         <v>0.54000000000000026</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A67" s="62" t="s">
         <v>127</v>
       </c>
@@ -8532,7 +8532,7 @@
         <v>0.55000000000000027</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A68" s="62" t="s">
         <v>124</v>
       </c>
@@ -8583,7 +8583,7 @@
         <v>0.56000000000000028</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A69" s="62" t="s">
         <v>126</v>
       </c>
@@ -8631,7 +8631,7 @@
         <v>0.57000000000000028</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A70" s="62" t="s">
         <v>126</v>
       </c>
@@ -8679,7 +8679,7 @@
         <v>0.58000000000000029</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A71" s="62" t="s">
         <v>126</v>
       </c>
@@ -8729,7 +8729,7 @@
         <v>0.5900000000000003</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A72" s="62" t="s">
         <v>127</v>
       </c>
@@ -8780,7 +8780,7 @@
         <v>0.60000000000000031</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A73" s="62" t="s">
         <v>124</v>
       </c>
@@ -8831,7 +8831,7 @@
         <v>0.61000000000000032</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A74" s="62" t="s">
         <v>126</v>
       </c>
@@ -8882,7 +8882,7 @@
         <v>0.62000000000000033</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A75" s="62" t="s">
         <v>126</v>
       </c>
@@ -8894,7 +8894,7 @@
         <v>222</v>
       </c>
       <c r="E75" s="172" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="F75" s="104">
         <v>8.6999999999999994E-3</v>
@@ -8935,7 +8935,7 @@
         <v>0.63000000000000034</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A76" s="62" t="s">
         <v>126</v>
       </c>
@@ -8985,10 +8985,10 @@
         <v>0.64000000000000035</v>
       </c>
       <c r="P76" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A77" s="62" t="s">
         <v>127</v>
       </c>
@@ -9038,7 +9038,7 @@
         <v>0.65000000000000036</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A78" s="62" t="s">
         <v>124</v>
       </c>
@@ -9089,7 +9089,7 @@
         <v>0.66000000000000036</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A79" s="62" t="s">
         <v>126</v>
       </c>
@@ -9139,7 +9139,7 @@
         <v>0.67000000000000037</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A80" s="62" t="s">
         <v>126</v>
       </c>
@@ -9189,7 +9189,7 @@
         <v>0.68000000000000038</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" s="125" t="s">
         <v>126</v>
       </c>
@@ -9239,7 +9239,7 @@
         <v>0.69000000000000039</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" s="125"/>
       <c r="B82" s="36"/>
       <c r="C82" s="36" t="s">
@@ -9288,7 +9288,7 @@
         <v>0.7000000000000004</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" s="125"/>
       <c r="B83" s="36"/>
       <c r="C83" s="36" t="s">
@@ -9337,7 +9337,7 @@
         <v>0.71000000000000041</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" s="125"/>
       <c r="B84" s="36"/>
       <c r="C84" s="36" t="s">
@@ -9386,7 +9386,7 @@
         <v>0.72000000000000042</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" s="125"/>
       <c r="B85" s="36"/>
       <c r="C85" s="36" t="s">
@@ -9435,7 +9435,7 @@
         <v>0.73000000000000043</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" s="125"/>
       <c r="B86" s="36"/>
       <c r="C86" s="36" t="s">
@@ -9484,10 +9484,10 @@
         <v>0.74000000000000044</v>
       </c>
       <c r="P86" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" s="125"/>
       <c r="B87" s="36"/>
       <c r="C87" s="36" t="s">
@@ -9533,7 +9533,7 @@
         <v>0.75000000000000044</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" s="125"/>
       <c r="B88" s="36"/>
       <c r="C88" s="36" t="s">
@@ -9582,7 +9582,7 @@
         <v>0.76000000000000045</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" s="125"/>
       <c r="B89" s="36"/>
       <c r="C89" s="36" t="s">
@@ -9631,7 +9631,7 @@
         <v>0.77000000000000046</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" s="125"/>
       <c r="B90" s="36"/>
       <c r="C90" s="36" t="s">
@@ -9677,7 +9677,7 @@
         <v>0.78000000000000047</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" s="125"/>
       <c r="B91" s="36"/>
       <c r="C91" s="36" t="s">
@@ -9723,7 +9723,7 @@
         <v>0.79000000000000048</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" s="125"/>
       <c r="B92" s="36"/>
       <c r="C92" s="36" t="s">
@@ -9772,7 +9772,7 @@
         <v>0.80000000000000049</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" s="125"/>
       <c r="B93" s="36"/>
       <c r="C93" s="36" t="s">
@@ -9821,7 +9821,7 @@
         <v>0.8100000000000005</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" s="125"/>
       <c r="B94" s="36"/>
       <c r="C94" s="36" t="s">
@@ -9870,7 +9870,7 @@
         <v>0.82000000000000051</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" s="125"/>
       <c r="B95" s="36"/>
       <c r="C95" s="36" t="s">
@@ -9919,7 +9919,7 @@
         <v>0.83000000000000052</v>
       </c>
     </row>
-    <row r="96" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="125"/>
       <c r="B96" s="36"/>
       <c r="C96" s="36" t="s">
@@ -9968,7 +9968,7 @@
         <v>0.84000000000000052</v>
       </c>
     </row>
-    <row r="97" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="125"/>
       <c r="B97" s="36"/>
       <c r="C97" s="36" t="s">
@@ -10017,7 +10017,7 @@
         <v>0.85000000000000053</v>
       </c>
     </row>
-    <row r="98" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="125"/>
       <c r="B98" s="36"/>
       <c r="C98" s="36" t="s">
@@ -10066,7 +10066,7 @@
         <v>0.86000000000000054</v>
       </c>
     </row>
-    <row r="99" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="125"/>
       <c r="B99" s="36"/>
       <c r="C99" s="36" t="s">
@@ -10112,7 +10112,7 @@
         <v>0.87000000000000055</v>
       </c>
     </row>
-    <row r="100" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="125"/>
       <c r="B100" s="36"/>
       <c r="C100" s="36" t="s">
@@ -10158,7 +10158,7 @@
         <v>0.88000000000000056</v>
       </c>
     </row>
-    <row r="101" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="125"/>
       <c r="B101" s="36"/>
       <c r="C101" s="36" t="s">
@@ -10206,7 +10206,7 @@
         <v>0.89000000000000057</v>
       </c>
     </row>
-    <row r="102" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="125"/>
       <c r="B102" s="36"/>
       <c r="C102" s="36" t="s">
@@ -10254,7 +10254,7 @@
         <v>0.90000000000000058</v>
       </c>
     </row>
-    <row r="103" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="125"/>
       <c r="B103" s="36"/>
       <c r="C103" s="36" t="s">
@@ -10303,7 +10303,7 @@
         <v>0.91000000000000059</v>
       </c>
     </row>
-    <row r="104" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="125"/>
       <c r="B104" s="36"/>
       <c r="C104" s="36" t="s">
@@ -10352,7 +10352,7 @@
         <v>0.9200000000000006</v>
       </c>
     </row>
-    <row r="105" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="125"/>
       <c r="B105" s="36"/>
       <c r="C105" s="36" t="s">
@@ -10401,7 +10401,7 @@
         <v>0.9300000000000006</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" s="125"/>
       <c r="B106" s="36"/>
       <c r="C106" s="36" t="s">
@@ -10447,7 +10447,7 @@
         <v>0.94000000000000061</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" s="125"/>
       <c r="B107" s="36"/>
       <c r="C107" s="36" t="s">
@@ -10496,7 +10496,7 @@
         <v>0.95000000000000062</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" s="125"/>
       <c r="B108" s="36"/>
       <c r="C108" s="36" t="s">
@@ -10545,7 +10545,7 @@
         <v>0.96000000000000063</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" s="125"/>
       <c r="B109" s="36"/>
       <c r="C109" s="36" t="s">
@@ -10594,7 +10594,7 @@
         <v>0.97000000000000064</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" s="125"/>
       <c r="B110" s="36"/>
       <c r="C110" s="36" t="s">
@@ -10643,7 +10643,7 @@
         <v>0.98000000000000065</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" s="125"/>
       <c r="B111" s="36"/>
       <c r="C111" s="36" t="s">
@@ -10692,7 +10692,7 @@
         <v>0.99000000000000066</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" s="125"/>
       <c r="B112" s="36"/>
       <c r="C112" s="36" t="s">
@@ -10741,7 +10741,7 @@
         <v>1.0000000000000007</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" s="148"/>
       <c r="B113" s="36"/>
       <c r="C113" s="36" t="s">
@@ -10790,7 +10790,7 @@
         <v>1.0100000000000007</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" s="148"/>
       <c r="B114" s="36"/>
       <c r="C114" s="36" t="s">
@@ -10839,7 +10839,7 @@
         <v>1.0200000000000007</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" s="148"/>
       <c r="B115" s="36"/>
       <c r="C115" s="36" t="s">
@@ -10888,7 +10888,7 @@
         <v>1.0300000000000007</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" s="148"/>
       <c r="B116" s="36"/>
       <c r="C116" s="36" t="s">
@@ -10937,7 +10937,7 @@
         <v>1.0400000000000007</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" s="148"/>
       <c r="B117" s="36"/>
       <c r="C117" s="36" t="s">
@@ -10983,7 +10983,7 @@
         <v>1.0500000000000007</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" s="148"/>
       <c r="B118" s="36"/>
       <c r="C118" s="36" t="s">
@@ -11032,7 +11032,7 @@
         <v>1.0600000000000007</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" s="148"/>
       <c r="B119" s="36"/>
       <c r="C119" s="36" t="s">
@@ -11081,7 +11081,7 @@
         <v>1.0700000000000007</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" s="148"/>
       <c r="B120" s="36"/>
       <c r="C120" s="36" t="s">
@@ -11130,7 +11130,7 @@
         <v>1.0800000000000007</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" s="148"/>
       <c r="B121" s="36"/>
       <c r="C121" s="36" t="s">
@@ -11179,7 +11179,7 @@
         <v>1.0900000000000007</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" s="148"/>
       <c r="B122" s="36"/>
       <c r="C122" s="36" t="s">
@@ -11228,7 +11228,7 @@
         <v>1.1000000000000008</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" s="148"/>
       <c r="B123" s="36"/>
       <c r="C123" s="36" t="s">
@@ -11277,7 +11277,7 @@
         <v>1.1100000000000008</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" s="148" t="s">
         <v>27</v>
       </c>
@@ -11328,7 +11328,7 @@
         <v>1.1200000000000008</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" s="148" t="s">
         <v>27</v>
       </c>
@@ -11379,7 +11379,7 @@
         <v>1.1300000000000008</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" s="56" t="s">
         <v>27</v>
       </c>
@@ -11397,7 +11397,7 @@
       <c r="M126" s="5"/>
       <c r="N126" s="9"/>
     </row>
-    <row r="127" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="28"/>
       <c r="B127" s="28"/>
       <c r="C127" s="28"/>
@@ -11438,41 +11438,41 @@
       </c>
       <c r="P127" s="64"/>
     </row>
-    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="K128" s="66">
         <f>K127-L1</f>
         <v>1240893.8416399993</v>
       </c>
     </row>
-    <row r="129" spans="3:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C129" s="195"/>
-      <c r="D129" s="195"/>
-      <c r="E129" s="195"/>
-      <c r="F129" s="195"/>
-      <c r="G129" s="195"/>
-      <c r="H129" s="195"/>
-      <c r="I129" s="195"/>
-      <c r="J129" s="195"/>
-      <c r="K129" s="195"/>
-      <c r="L129" s="195"/>
-      <c r="M129" s="195"/>
-      <c r="N129" s="195"/>
-    </row>
-    <row r="130" spans="3:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C130" s="195"/>
-      <c r="D130" s="195"/>
-      <c r="E130" s="195"/>
-      <c r="F130" s="195"/>
-      <c r="G130" s="195"/>
-      <c r="H130" s="195"/>
-      <c r="I130" s="195"/>
-      <c r="J130" s="195"/>
-      <c r="K130" s="195"/>
-      <c r="L130" s="195"/>
-      <c r="M130" s="195"/>
-      <c r="N130" s="195"/>
-    </row>
-    <row r="131" spans="3:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="3:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C129" s="199"/>
+      <c r="D129" s="199"/>
+      <c r="E129" s="199"/>
+      <c r="F129" s="199"/>
+      <c r="G129" s="199"/>
+      <c r="H129" s="199"/>
+      <c r="I129" s="199"/>
+      <c r="J129" s="199"/>
+      <c r="K129" s="199"/>
+      <c r="L129" s="199"/>
+      <c r="M129" s="199"/>
+      <c r="N129" s="199"/>
+    </row>
+    <row r="130" spans="3:16" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C130" s="199"/>
+      <c r="D130" s="199"/>
+      <c r="E130" s="199"/>
+      <c r="F130" s="199"/>
+      <c r="G130" s="199"/>
+      <c r="H130" s="199"/>
+      <c r="I130" s="199"/>
+      <c r="J130" s="199"/>
+      <c r="K130" s="199"/>
+      <c r="L130" s="199"/>
+      <c r="M130" s="199"/>
+      <c r="N130" s="199"/>
+    </row>
+    <row r="131" spans="3:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="87"/>
       <c r="D131" s="87"/>
       <c r="E131" s="87"/>
@@ -11486,121 +11486,121 @@
       <c r="M131" s="87"/>
       <c r="N131" s="87"/>
     </row>
-    <row r="132" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C132" s="195" t="s">
+    <row r="132" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C132" s="199" t="s">
         <v>269</v>
       </c>
-      <c r="D132" s="195"/>
-      <c r="E132" s="195"/>
-      <c r="F132" s="195"/>
-      <c r="G132" s="195"/>
-      <c r="H132" s="195"/>
-      <c r="I132" s="195"/>
-      <c r="J132" s="195"/>
-      <c r="K132" s="195"/>
-      <c r="L132" s="195"/>
-      <c r="M132" s="195"/>
-      <c r="N132" s="195"/>
-    </row>
-    <row r="133" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C133" s="195"/>
-      <c r="D133" s="195"/>
-      <c r="E133" s="195"/>
-      <c r="F133" s="195"/>
-      <c r="G133" s="195"/>
-      <c r="H133" s="195"/>
-      <c r="I133" s="195"/>
-      <c r="J133" s="195"/>
-      <c r="K133" s="195"/>
-      <c r="L133" s="195"/>
-      <c r="M133" s="195"/>
-      <c r="N133" s="195"/>
-    </row>
-    <row r="134" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C134" s="195"/>
-      <c r="D134" s="195"/>
-      <c r="E134" s="195"/>
-      <c r="F134" s="195"/>
-      <c r="G134" s="195"/>
-      <c r="H134" s="195"/>
-      <c r="I134" s="195"/>
-      <c r="J134" s="195"/>
-      <c r="K134" s="195"/>
-      <c r="L134" s="195"/>
-      <c r="M134" s="195"/>
-      <c r="N134" s="195"/>
-    </row>
-    <row r="135" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C135" s="195"/>
-      <c r="D135" s="195"/>
-      <c r="E135" s="195"/>
-      <c r="F135" s="195"/>
-      <c r="G135" s="195"/>
-      <c r="H135" s="195"/>
-      <c r="I135" s="195"/>
-      <c r="J135" s="195"/>
-      <c r="K135" s="195"/>
-      <c r="L135" s="195"/>
-      <c r="M135" s="195"/>
-      <c r="N135" s="195"/>
-    </row>
-    <row r="136" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C136" s="195"/>
-      <c r="D136" s="195"/>
-      <c r="E136" s="195"/>
-      <c r="F136" s="195"/>
-      <c r="G136" s="195"/>
-      <c r="H136" s="195"/>
-      <c r="I136" s="195"/>
-      <c r="J136" s="195"/>
-      <c r="K136" s="195"/>
-      <c r="L136" s="195"/>
-      <c r="M136" s="195"/>
-      <c r="N136" s="195"/>
-    </row>
-    <row r="137" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C137" s="195"/>
-      <c r="D137" s="195"/>
-      <c r="E137" s="195"/>
-      <c r="F137" s="195"/>
-      <c r="G137" s="195"/>
-      <c r="H137" s="195"/>
-      <c r="I137" s="195"/>
-      <c r="J137" s="195"/>
-      <c r="K137" s="195"/>
-      <c r="L137" s="195"/>
-      <c r="M137" s="195"/>
-      <c r="N137" s="195"/>
-    </row>
-    <row r="138" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C138" s="195"/>
-      <c r="D138" s="195"/>
-      <c r="E138" s="195"/>
-      <c r="F138" s="195"/>
-      <c r="G138" s="195"/>
-      <c r="H138" s="195"/>
-      <c r="I138" s="195"/>
-      <c r="J138" s="195"/>
-      <c r="K138" s="195"/>
-      <c r="L138" s="195"/>
-      <c r="M138" s="195"/>
-      <c r="N138" s="195"/>
-    </row>
-    <row r="139" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C139" s="195"/>
-      <c r="D139" s="195"/>
-      <c r="E139" s="195"/>
-      <c r="F139" s="195"/>
-      <c r="G139" s="195"/>
-      <c r="H139" s="195"/>
-      <c r="I139" s="195"/>
-      <c r="J139" s="195"/>
-      <c r="K139" s="195"/>
-      <c r="L139" s="195"/>
-      <c r="M139" s="195"/>
-      <c r="N139" s="195"/>
-    </row>
-    <row r="140" spans="3:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D132" s="199"/>
+      <c r="E132" s="199"/>
+      <c r="F132" s="199"/>
+      <c r="G132" s="199"/>
+      <c r="H132" s="199"/>
+      <c r="I132" s="199"/>
+      <c r="J132" s="199"/>
+      <c r="K132" s="199"/>
+      <c r="L132" s="199"/>
+      <c r="M132" s="199"/>
+      <c r="N132" s="199"/>
+    </row>
+    <row r="133" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C133" s="199"/>
+      <c r="D133" s="199"/>
+      <c r="E133" s="199"/>
+      <c r="F133" s="199"/>
+      <c r="G133" s="199"/>
+      <c r="H133" s="199"/>
+      <c r="I133" s="199"/>
+      <c r="J133" s="199"/>
+      <c r="K133" s="199"/>
+      <c r="L133" s="199"/>
+      <c r="M133" s="199"/>
+      <c r="N133" s="199"/>
+    </row>
+    <row r="134" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C134" s="199"/>
+      <c r="D134" s="199"/>
+      <c r="E134" s="199"/>
+      <c r="F134" s="199"/>
+      <c r="G134" s="199"/>
+      <c r="H134" s="199"/>
+      <c r="I134" s="199"/>
+      <c r="J134" s="199"/>
+      <c r="K134" s="199"/>
+      <c r="L134" s="199"/>
+      <c r="M134" s="199"/>
+      <c r="N134" s="199"/>
+    </row>
+    <row r="135" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C135" s="199"/>
+      <c r="D135" s="199"/>
+      <c r="E135" s="199"/>
+      <c r="F135" s="199"/>
+      <c r="G135" s="199"/>
+      <c r="H135" s="199"/>
+      <c r="I135" s="199"/>
+      <c r="J135" s="199"/>
+      <c r="K135" s="199"/>
+      <c r="L135" s="199"/>
+      <c r="M135" s="199"/>
+      <c r="N135" s="199"/>
+    </row>
+    <row r="136" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C136" s="199"/>
+      <c r="D136" s="199"/>
+      <c r="E136" s="199"/>
+      <c r="F136" s="199"/>
+      <c r="G136" s="199"/>
+      <c r="H136" s="199"/>
+      <c r="I136" s="199"/>
+      <c r="J136" s="199"/>
+      <c r="K136" s="199"/>
+      <c r="L136" s="199"/>
+      <c r="M136" s="199"/>
+      <c r="N136" s="199"/>
+    </row>
+    <row r="137" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C137" s="199"/>
+      <c r="D137" s="199"/>
+      <c r="E137" s="199"/>
+      <c r="F137" s="199"/>
+      <c r="G137" s="199"/>
+      <c r="H137" s="199"/>
+      <c r="I137" s="199"/>
+      <c r="J137" s="199"/>
+      <c r="K137" s="199"/>
+      <c r="L137" s="199"/>
+      <c r="M137" s="199"/>
+      <c r="N137" s="199"/>
+    </row>
+    <row r="138" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C138" s="199"/>
+      <c r="D138" s="199"/>
+      <c r="E138" s="199"/>
+      <c r="F138" s="199"/>
+      <c r="G138" s="199"/>
+      <c r="H138" s="199"/>
+      <c r="I138" s="199"/>
+      <c r="J138" s="199"/>
+      <c r="K138" s="199"/>
+      <c r="L138" s="199"/>
+      <c r="M138" s="199"/>
+      <c r="N138" s="199"/>
+    </row>
+    <row r="139" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C139" s="199"/>
+      <c r="D139" s="199"/>
+      <c r="E139" s="199"/>
+      <c r="F139" s="199"/>
+      <c r="G139" s="199"/>
+      <c r="H139" s="199"/>
+      <c r="I139" s="199"/>
+      <c r="J139" s="199"/>
+      <c r="K139" s="199"/>
+      <c r="L139" s="199"/>
+      <c r="M139" s="199"/>
+      <c r="N139" s="199"/>
+    </row>
+    <row r="140" spans="3:16" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="87"/>
       <c r="D140" s="87"/>
       <c r="E140" s="87"/>
@@ -11614,7 +11614,7 @@
       <c r="M140" s="87"/>
       <c r="N140" s="87"/>
     </row>
-    <row r="141" spans="3:16" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="3:16" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="87"/>
       <c r="D141" s="87"/>
       <c r="E141" s="87"/>
@@ -11628,118 +11628,112 @@
       <c r="M141" s="87"/>
       <c r="N141" s="87"/>
     </row>
-    <row r="142" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C142" s="194" t="s">
+    <row r="142" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C142" s="198" t="s">
         <v>268</v>
       </c>
-      <c r="D142" s="194"/>
-      <c r="E142" s="194"/>
-      <c r="F142" s="194"/>
-      <c r="G142" s="194"/>
-      <c r="H142" s="194"/>
-      <c r="I142" s="194"/>
-      <c r="J142" s="194"/>
-      <c r="K142" s="194"/>
-      <c r="L142" s="194"/>
-      <c r="M142" s="194"/>
-      <c r="N142" s="194"/>
-    </row>
-    <row r="143" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C143" s="194"/>
-      <c r="D143" s="194"/>
-      <c r="E143" s="194"/>
-      <c r="F143" s="194"/>
-      <c r="G143" s="194"/>
-      <c r="H143" s="194"/>
-      <c r="I143" s="194"/>
-      <c r="J143" s="194"/>
-      <c r="K143" s="194"/>
-      <c r="L143" s="194"/>
-      <c r="M143" s="194"/>
-      <c r="N143" s="194"/>
-    </row>
-    <row r="144" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C144" s="194"/>
-      <c r="D144" s="194"/>
-      <c r="E144" s="194"/>
-      <c r="F144" s="194"/>
-      <c r="G144" s="194"/>
-      <c r="H144" s="194"/>
-      <c r="I144" s="194"/>
-      <c r="J144" s="194"/>
-      <c r="K144" s="194"/>
-      <c r="L144" s="194"/>
-      <c r="M144" s="194"/>
-      <c r="N144" s="194"/>
+      <c r="D142" s="198"/>
+      <c r="E142" s="198"/>
+      <c r="F142" s="198"/>
+      <c r="G142" s="198"/>
+      <c r="H142" s="198"/>
+      <c r="I142" s="198"/>
+      <c r="J142" s="198"/>
+      <c r="K142" s="198"/>
+      <c r="L142" s="198"/>
+      <c r="M142" s="198"/>
+      <c r="N142" s="198"/>
+    </row>
+    <row r="143" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C143" s="198"/>
+      <c r="D143" s="198"/>
+      <c r="E143" s="198"/>
+      <c r="F143" s="198"/>
+      <c r="G143" s="198"/>
+      <c r="H143" s="198"/>
+      <c r="I143" s="198"/>
+      <c r="J143" s="198"/>
+      <c r="K143" s="198"/>
+      <c r="L143" s="198"/>
+      <c r="M143" s="198"/>
+      <c r="N143" s="198"/>
+    </row>
+    <row r="144" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C144" s="198"/>
+      <c r="D144" s="198"/>
+      <c r="E144" s="198"/>
+      <c r="F144" s="198"/>
+      <c r="G144" s="198"/>
+      <c r="H144" s="198"/>
+      <c r="I144" s="198"/>
+      <c r="J144" s="198"/>
+      <c r="K144" s="198"/>
+      <c r="L144" s="198"/>
+      <c r="M144" s="198"/>
+      <c r="N144" s="198"/>
       <c r="P144" s="95">
         <f>L1-K127</f>
         <v>-1240893.8416399993</v>
       </c>
     </row>
-    <row r="145" spans="3:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C145" s="194"/>
-      <c r="D145" s="194"/>
-      <c r="E145" s="194"/>
-      <c r="F145" s="194"/>
-      <c r="G145" s="194"/>
-      <c r="H145" s="194"/>
-      <c r="I145" s="194"/>
-      <c r="J145" s="194"/>
-      <c r="K145" s="194"/>
-      <c r="L145" s="194"/>
-      <c r="M145" s="194"/>
-      <c r="N145" s="194"/>
-    </row>
-    <row r="146" spans="3:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C146" s="194"/>
-      <c r="D146" s="194"/>
-      <c r="E146" s="194"/>
-      <c r="F146" s="194"/>
-      <c r="G146" s="194"/>
-      <c r="H146" s="194"/>
-      <c r="I146" s="194"/>
-      <c r="J146" s="194"/>
-      <c r="K146" s="194"/>
-      <c r="L146" s="194"/>
-      <c r="M146" s="194"/>
-      <c r="N146" s="194"/>
-    </row>
-    <row r="147" spans="3:14" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C147" s="194"/>
-      <c r="D147" s="194"/>
-      <c r="E147" s="194"/>
-      <c r="F147" s="194"/>
-      <c r="G147" s="194"/>
-      <c r="H147" s="194"/>
-      <c r="I147" s="194"/>
-      <c r="J147" s="194"/>
-      <c r="K147" s="194"/>
-      <c r="L147" s="194"/>
-      <c r="M147" s="194"/>
-      <c r="N147" s="194"/>
-    </row>
-    <row r="148" spans="3:14" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C148" s="194"/>
-      <c r="D148" s="194"/>
-      <c r="E148" s="194"/>
-      <c r="F148" s="194"/>
-      <c r="G148" s="194"/>
-      <c r="H148" s="194"/>
-      <c r="I148" s="194"/>
-      <c r="J148" s="194"/>
-      <c r="K148" s="194"/>
-      <c r="L148" s="194"/>
-      <c r="M148" s="194"/>
-      <c r="N148" s="194"/>
+    <row r="145" spans="3:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C145" s="198"/>
+      <c r="D145" s="198"/>
+      <c r="E145" s="198"/>
+      <c r="F145" s="198"/>
+      <c r="G145" s="198"/>
+      <c r="H145" s="198"/>
+      <c r="I145" s="198"/>
+      <c r="J145" s="198"/>
+      <c r="K145" s="198"/>
+      <c r="L145" s="198"/>
+      <c r="M145" s="198"/>
+      <c r="N145" s="198"/>
+    </row>
+    <row r="146" spans="3:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C146" s="198"/>
+      <c r="D146" s="198"/>
+      <c r="E146" s="198"/>
+      <c r="F146" s="198"/>
+      <c r="G146" s="198"/>
+      <c r="H146" s="198"/>
+      <c r="I146" s="198"/>
+      <c r="J146" s="198"/>
+      <c r="K146" s="198"/>
+      <c r="L146" s="198"/>
+      <c r="M146" s="198"/>
+      <c r="N146" s="198"/>
+    </row>
+    <row r="147" spans="3:14" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C147" s="198"/>
+      <c r="D147" s="198"/>
+      <c r="E147" s="198"/>
+      <c r="F147" s="198"/>
+      <c r="G147" s="198"/>
+      <c r="H147" s="198"/>
+      <c r="I147" s="198"/>
+      <c r="J147" s="198"/>
+      <c r="K147" s="198"/>
+      <c r="L147" s="198"/>
+      <c r="M147" s="198"/>
+      <c r="N147" s="198"/>
+    </row>
+    <row r="148" spans="3:14" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C148" s="198"/>
+      <c r="D148" s="198"/>
+      <c r="E148" s="198"/>
+      <c r="F148" s="198"/>
+      <c r="G148" s="198"/>
+      <c r="H148" s="198"/>
+      <c r="I148" s="198"/>
+      <c r="J148" s="198"/>
+      <c r="K148" s="198"/>
+      <c r="L148" s="198"/>
+      <c r="M148" s="198"/>
+      <c r="N148" s="198"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="F5:F7"/>
-    <mergeCell ref="E5:E7"/>
     <mergeCell ref="Q8:R9"/>
     <mergeCell ref="G5:G7"/>
     <mergeCell ref="C142:N148"/>
@@ -11753,6 +11747,12 @@
     <mergeCell ref="C132:N139"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="E5:E7"/>
   </mergeCells>
   <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11764,11 +11764,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7365EFC1-5C09-4380-B9A2-A73102AE2F7A}">
   <dimension ref="B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="179" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -11779,90 +11779,90 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8B3D07-243A-48F3-942B-AB44D486DEC8}">
   <dimension ref="C4:D14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C4" s="209" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="D4" s="209"/>
     </row>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C5" s="177">
         <v>52141.08</v>
       </c>
       <c r="D5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C6" s="177">
         <v>67140.100000000006</v>
       </c>
       <c r="D6" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C7" s="177">
         <v>52121.11</v>
       </c>
       <c r="D7" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C8" s="177">
         <v>67885.119999999995</v>
       </c>
       <c r="D8" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C9" s="177">
         <v>67140.160000000003</v>
       </c>
       <c r="D9" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C10" s="177">
         <v>62141.17</v>
       </c>
       <c r="D10" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C11" s="177">
         <v>67855.179999999993</v>
       </c>
       <c r="D11" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C12" s="177">
         <v>62141.23</v>
       </c>
       <c r="D12" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C13" s="177">
         <v>67855.240000000005</v>
       </c>
       <c r="D13" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C14" s="177">
         <f>SUM(C5:C13)</f>
         <v>566420.39</v>

</xml_diff>